<commit_message>
feat(unit-04): build participant import, event flags and credentials
Add the participant module (backend modules/participant, frontend
features/participant) mirroring the question import, with the
individualEvent/teamEvent flags migration
(20261011000000_add_participant_event_flags) and the ParticipantPanel
wired into the competition setup screen. Filter the individual
ranking and round-participation reads on individualEvent so
team-only participants are not dealt into individual rounds. Teams
are deferred (U-102); no Team row is written. Spec approved
2026-10-11; docs, decisions and sample file updated to match.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/context/samples/选手信息.xlsx
+++ b/context/samples/选手信息.xlsx
@@ -3,8 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\sudoku\context\samples\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="29400" windowHeight="12560"/>
+    <workbookView windowWidth="18350" windowHeight="6880"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="24">
   <si>
     <t>比赛名称</t>
   </si>
@@ -65,7 +70,40 @@
     <t>备注</t>
   </si>
   <si>
+    <t>test2</t>
+  </si>
+  <si>
+    <t>张三</t>
+  </si>
+  <si>
+    <t>浙江</t>
+  </si>
+  <si>
+    <t>杭州</t>
+  </si>
+  <si>
+    <t>西湖</t>
+  </si>
+  <si>
+    <t>浙江科技大学</t>
+  </si>
+  <si>
+    <t>G12</t>
+  </si>
+  <si>
     <t>个人赛团队赛参加填写1，未参加空白或者是2</t>
+  </si>
+  <si>
+    <t>李四</t>
+  </si>
+  <si>
+    <t>湖州</t>
+  </si>
+  <si>
+    <t>安吉</t>
+  </si>
+  <si>
+    <t>刘一</t>
   </si>
 </sst>
 </file>
@@ -73,10 +111,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="20">
     <font>
@@ -536,19 +574,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1210,8 +1248,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:L2"/>
-  <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelRow="1"/>
+  <dimension ref="A1:L4"/>
+  <sheetFormatPr defaultColWidth="9.22727272727273" defaultRowHeight="14" outlineLevelRow="3"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" t="s">
@@ -1252,8 +1290,102 @@
       </c>
     </row>
     <row r="2" spans="1:12">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2">
+        <v>5</v>
+      </c>
+      <c r="E2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
       <c r="L2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" t="s">
         <v>12</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3">
+        <v>4</v>
+      </c>
+      <c r="E3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I3" t="s">
+        <v>18</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4">
+        <v>5</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I4" t="s">
+        <v>18</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>